<commit_message>
feat: update aux local crawl 6/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10223,33 +10223,61 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C7" s="59" t="n"/>
-      <c r="D7" s="168" t="n"/>
-      <c r="E7" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C7" s="59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D7" s="168" t="n">
+        <v>46270.02244059028</v>
+      </c>
+      <c r="E7" s="168" t="n">
+        <v>46270.55446297453</v>
+      </c>
       <c r="F7" s="169">
         <f>IF(AND(D7&lt;&gt;"",E7&lt;&gt;""),(E7-D7)*24,"")</f>
         <v/>
       </c>
-      <c r="G7" s="170" t="n"/>
-      <c r="H7" s="170" t="n"/>
-      <c r="I7" s="170" t="n"/>
-      <c r="J7" s="170" t="n"/>
-      <c r="K7" s="170" t="n"/>
-      <c r="L7" s="170" t="n"/>
-      <c r="M7" s="170" t="n"/>
-      <c r="N7" s="170" t="n"/>
+      <c r="G7" s="170" t="n">
+        <v>2478</v>
+      </c>
+      <c r="H7" s="170" t="n">
+        <v>2478</v>
+      </c>
+      <c r="I7" s="170" t="n">
+        <v>2190</v>
+      </c>
+      <c r="J7" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="170" t="n">
+        <v>253</v>
+      </c>
+      <c r="L7" s="170" t="n">
+        <v>21</v>
+      </c>
+      <c r="M7" s="170" t="n">
+        <v>14</v>
+      </c>
+      <c r="N7" s="170" t="n">
+        <v>20413</v>
+      </c>
       <c r="O7" s="170" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="P7" s="59" t="inlineStr">
         <is>
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q7" s="59" t="n"/>
+      <c r="Q7" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 4 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="167" t="n">
@@ -10257,24 +10285,48 @@
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C8" s="59" t="n"/>
-      <c r="D8" s="168" t="n"/>
-      <c r="E8" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D8" s="168" t="n">
+        <v>46271.02421355324</v>
+      </c>
+      <c r="E8" s="168" t="n">
+        <v>46271.84374591397</v>
+      </c>
       <c r="F8" s="169">
         <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),(E8-D8)*24,"")</f>
         <v/>
       </c>
-      <c r="G8" s="170" t="n"/>
-      <c r="H8" s="170" t="n"/>
-      <c r="I8" s="170" t="n"/>
-      <c r="J8" s="170" t="n"/>
-      <c r="K8" s="170" t="n"/>
-      <c r="L8" s="170" t="n"/>
-      <c r="M8" s="170" t="n"/>
-      <c r="N8" s="170" t="n"/>
+      <c r="G8" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H8" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I8" s="170" t="n">
+        <v>3185</v>
+      </c>
+      <c r="J8" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="170" t="n">
+        <v>305</v>
+      </c>
+      <c r="L8" s="170" t="n">
+        <v>30</v>
+      </c>
+      <c r="M8" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N8" s="170" t="n">
+        <v>29179</v>
+      </c>
       <c r="O8" s="170" t="n">
         <v>10</v>
       </c>
@@ -10283,7 +10335,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q8" s="59" t="n"/>
+      <c r="Q8" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 5 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux local crawl 7/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10297,7 +10297,7 @@
         <v>46271.02421355324</v>
       </c>
       <c r="E8" s="168" t="n">
-        <v>46271.84374591397</v>
+        <v>46271.84374591435</v>
       </c>
       <c r="F8" s="169">
         <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),(E8-D8)*24,"")</f>
@@ -10347,24 +10347,48 @@
       </c>
       <c r="B9" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C9" s="59" t="n"/>
-      <c r="D9" s="168" t="n"/>
-      <c r="E9" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C9" s="59" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D9" s="168" t="n">
+        <v>46272.02454877315</v>
+      </c>
+      <c r="E9" s="168" t="n">
+        <v>46272.81493315812</v>
+      </c>
       <c r="F9" s="169">
         <f>IF(AND(D9&lt;&gt;"",E9&lt;&gt;""),(E9-D9)*24,"")</f>
         <v/>
       </c>
-      <c r="G9" s="170" t="n"/>
-      <c r="H9" s="170" t="n"/>
-      <c r="I9" s="170" t="n"/>
-      <c r="J9" s="170" t="n"/>
-      <c r="K9" s="170" t="n"/>
-      <c r="L9" s="170" t="n"/>
-      <c r="M9" s="170" t="n"/>
-      <c r="N9" s="170" t="n"/>
+      <c r="G9" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H9" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I9" s="170" t="n">
+        <v>3177</v>
+      </c>
+      <c r="J9" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="170" t="n">
+        <v>313</v>
+      </c>
+      <c r="L9" s="170" t="n">
+        <v>30</v>
+      </c>
+      <c r="M9" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N9" s="170" t="n">
+        <v>28420</v>
+      </c>
       <c r="O9" s="170" t="n">
         <v>10</v>
       </c>
@@ -10373,7 +10397,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q9" s="59" t="n"/>
+      <c r="Q9" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 6 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 8/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10359,7 +10359,7 @@
         <v>46272.02454877315</v>
       </c>
       <c r="E9" s="168" t="n">
-        <v>46272.81493315812</v>
+        <v>46272.81493315972</v>
       </c>
       <c r="F9" s="169">
         <f>IF(AND(D9&lt;&gt;"",E9&lt;&gt;""),(E9-D9)*24,"")</f>
@@ -10409,24 +10409,48 @@
       </c>
       <c r="B10" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C10" s="59" t="n"/>
-      <c r="D10" s="168" t="n"/>
-      <c r="E10" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D10" s="168" t="n">
+        <v>46273.02355465278</v>
+      </c>
+      <c r="E10" s="168" t="n">
+        <v>46273.82085170058</v>
+      </c>
       <c r="F10" s="169">
         <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),(E10-D10)*24,"")</f>
         <v/>
       </c>
-      <c r="G10" s="170" t="n"/>
-      <c r="H10" s="170" t="n"/>
-      <c r="I10" s="170" t="n"/>
-      <c r="J10" s="170" t="n"/>
-      <c r="K10" s="170" t="n"/>
-      <c r="L10" s="170" t="n"/>
-      <c r="M10" s="170" t="n"/>
-      <c r="N10" s="170" t="n"/>
+      <c r="G10" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H10" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I10" s="170" t="n">
+        <v>3174</v>
+      </c>
+      <c r="J10" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="170" t="n">
+        <v>306</v>
+      </c>
+      <c r="L10" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M10" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N10" s="170" t="n">
+        <v>29258</v>
+      </c>
       <c r="O10" s="170" t="n">
         <v>10</v>
       </c>
@@ -10435,7 +10459,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q10" s="59" t="n"/>
+      <c r="Q10" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 7 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 10/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10421,7 +10421,7 @@
         <v>46273.02355465278</v>
       </c>
       <c r="E10" s="168" t="n">
-        <v>46273.82085170058</v>
+        <v>46273.82085170139</v>
       </c>
       <c r="F10" s="169">
         <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),(E10-D10)*24,"")</f>
@@ -10471,24 +10471,48 @@
       </c>
       <c r="B11" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C11" s="59" t="n"/>
-      <c r="D11" s="168" t="n"/>
-      <c r="E11" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C11" s="59" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D11" s="168" t="n">
+        <v>46274.02572726852</v>
+      </c>
+      <c r="E11" s="168" t="n">
+        <v>46275.02770430457</v>
+      </c>
       <c r="F11" s="169">
         <f>IF(AND(D11&lt;&gt;"",E11&lt;&gt;""),(E11-D11)*24,"")</f>
         <v/>
       </c>
-      <c r="G11" s="170" t="n"/>
-      <c r="H11" s="170" t="n"/>
-      <c r="I11" s="170" t="n"/>
-      <c r="J11" s="170" t="n"/>
-      <c r="K11" s="170" t="n"/>
-      <c r="L11" s="170" t="n"/>
-      <c r="M11" s="170" t="n"/>
-      <c r="N11" s="170" t="n"/>
+      <c r="G11" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H11" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I11" s="170" t="n">
+        <v>3165</v>
+      </c>
+      <c r="J11" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="170" t="n">
+        <v>305</v>
+      </c>
+      <c r="L11" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="M11" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N11" s="170" t="n">
+        <v>29944</v>
+      </c>
       <c r="O11" s="170" t="n">
         <v>10</v>
       </c>
@@ -10497,7 +10521,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q11" s="59" t="n"/>
+      <c r="Q11" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 8 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="167" t="n">
@@ -10505,11 +10533,17 @@
       </c>
       <c r="B12" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C12" s="59" t="n"/>
-      <c r="D12" s="168" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D12" s="168" t="n">
+        <v>46275.02272983796</v>
+      </c>
       <c r="E12" s="168" t="n"/>
       <c r="F12" s="169">
         <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),(E12-D12)*24,"")</f>
@@ -10531,7 +10565,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q12" s="59" t="n"/>
+      <c r="Q12" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="167" t="n">

</xml_diff>

<commit_message>
feat: fix run scheduled automation
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10545,7 +10545,7 @@
         <v>46275.02272983796</v>
       </c>
       <c r="E12" s="168" t="n">
-        <v>46275.83740755328</v>
+        <v>46275.83740755787</v>
       </c>
       <c r="F12" s="169">
         <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),(E12-D12)*24,"")</f>
@@ -10595,24 +10595,48 @@
       </c>
       <c r="B13" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C13" s="59" t="n"/>
-      <c r="D13" s="168" t="n"/>
-      <c r="E13" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C13" s="59" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D13" s="168" t="n">
+        <v>46276.0238975</v>
+      </c>
+      <c r="E13" s="168" t="n">
+        <v>46276.85525002315</v>
+      </c>
       <c r="F13" s="169">
         <f>IF(AND(D13&lt;&gt;"",E13&lt;&gt;""),(E13-D13)*24,"")</f>
         <v/>
       </c>
-      <c r="G13" s="170" t="n"/>
-      <c r="H13" s="170" t="n"/>
-      <c r="I13" s="170" t="n"/>
-      <c r="J13" s="170" t="n"/>
-      <c r="K13" s="170" t="n"/>
-      <c r="L13" s="170" t="n"/>
-      <c r="M13" s="170" t="n"/>
-      <c r="N13" s="170" t="n"/>
+      <c r="G13" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H13" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I13" s="170" t="n">
+        <v>3174</v>
+      </c>
+      <c r="J13" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="170" t="n">
+        <v>316</v>
+      </c>
+      <c r="L13" s="170" t="n">
+        <v>30</v>
+      </c>
+      <c r="M13" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N13" s="170" t="n">
+        <v>30010</v>
+      </c>
       <c r="O13" s="170" t="n">
         <v>10</v>
       </c>
@@ -10621,7 +10645,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q13" s="59" t="n"/>
+      <c r="Q13" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 10 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="167" t="n">
@@ -10629,11 +10657,17 @@
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C14" s="59" t="n"/>
-      <c r="D14" s="168" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="C14" s="59" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D14" s="168" t="n">
+        <v>46277.02385240931</v>
+      </c>
       <c r="E14" s="168" t="n"/>
       <c r="F14" s="169">
         <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),(E14-D14)*24,"")</f>
@@ -10655,7 +10689,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q14" s="59" t="n"/>
+      <c r="Q14" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="167" t="n">

</xml_diff>